<commit_message>
Handle browser pages and verify all disputed spreadsheet rows
</commit_message>
<xml_diff>
--- a/out/result.xlsx
+++ b/out/result.xlsx
@@ -19,9 +19,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Строки'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Книги'!$A$1:$I$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Дубли'!$A$1:$F$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Спорные'!$A$1:$G$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Спорные'!$A$1:$G$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Задание 2'!$A$1:$M$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Рекомендации ИИ'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Рекомендации ИИ'!$A$1:$E$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -718,7 +718,7 @@
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr"/>
@@ -793,7 +793,7 @@
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S3" s="4" t="inlineStr"/>
@@ -860,14 +860,18 @@
       <c r="O4" s="4" t="inlineStr"/>
       <c r="P4" s="4" t="inlineStr"/>
       <c r="Q4" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R4" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>B5d524b</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -931,18 +935,14 @@
       <c r="O5" s="4" t="inlineStr"/>
       <c r="P5" s="4" t="inlineStr"/>
       <c r="Q5" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S5" s="4" t="inlineStr">
-        <is>
-          <t>B5d524b</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Название "ПРОМПТ SUNO.COM энциклопедия и полное руководство по составлению промпта." совпало, но автора из каталога (DIGITAL ZEN) на странице нет. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="S8" s="4" t="inlineStr"/>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S9" s="4" t="inlineStr"/>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="R10" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S10" s="4" t="inlineStr"/>
@@ -1610,11 +1610,11 @@
         </is>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>Название "Измена. Хочу твоего мужа" совпало, но автора из каталога (Ася Исай, Галина Колоскова, Мария Авенская) на странице нет. Нужна проверка человеком.</t>
+          <t>ИИ-проверка: Название совпадает, но указанный на странице автор Оксана Алексаева отсутствует среди кандидатов.</t>
         </is>
       </c>
       <c r="S14" s="3" t="inlineStr"/>
@@ -1831,18 +1831,14 @@
       <c r="O17" s="4" t="inlineStr"/>
       <c r="P17" s="4" t="inlineStr"/>
       <c r="Q17" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S17" s="4" t="inlineStr">
-        <is>
-          <t>B9bae6e</t>
-        </is>
-      </c>
+          <t>Сайт не ответил (Timeout).</t>
+        </is>
+      </c>
+      <c r="S17" s="4" t="inlineStr"/>
     </row>
     <row r="18" ht="58" customHeight="1">
       <c r="A18" s="4" t="n">
@@ -2066,7 +2062,7 @@
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Название "ПРОМПТ SUNO.COM энциклопедия и полное руководство по составлению промпта." совпало, но автора из каталога (DIGITAL ZEN) на странице нет. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr"/>
@@ -2522,7 +2518,7 @@
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr"/>
@@ -2593,7 +2589,7 @@
       </c>
       <c r="R27" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2, txt; чтение онлайн; кнопка скачивания.</t>
+          <t>ИИ-проверка: Название и автор (Хельга Дюран / Helga Duran) совпадают с каталогом, книга размещена с возможностью скачивания.</t>
         </is>
       </c>
       <c r="S27" s="4" t="inlineStr">
@@ -2739,18 +2735,14 @@
       <c r="O29" s="4" t="inlineStr"/>
       <c r="P29" s="4" t="inlineStr"/>
       <c r="Q29" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R29" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S29" s="4" t="inlineStr">
-        <is>
-          <t>B584abb</t>
-        </is>
-      </c>
+          <t>Название "Тарский горячий твой" совпало, но автора из каталога (Helga Duran) на странице нет. На странице указан автор: Daniella. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S29" s="4" t="inlineStr"/>
     </row>
     <row r="30" ht="58" customHeight="1">
       <c r="A30" s="4" t="n">
@@ -2897,7 +2889,7 @@
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Кармическая астрология | Книги по кармической астрологии</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Кармическая астрология | Книги по кармической астрологии</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr"/>
@@ -3122,7 +3114,7 @@
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S34" s="4" t="inlineStr"/>
@@ -3345,18 +3337,14 @@
       <c r="O37" s="4" t="inlineStr"/>
       <c r="P37" s="4" t="inlineStr"/>
       <c r="Q37" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R37" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S37" s="4" t="inlineStr">
-        <is>
-          <t>Bd7871a</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="58" customHeight="1">
       <c r="A38" s="4" t="n">
@@ -3424,7 +3412,7 @@
       </c>
       <c r="R38" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S38" s="4" t="inlineStr"/>
@@ -4099,11 +4087,11 @@
         </is>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R47" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: ОГЭ-2026 по английскому. Лайфхаки, фейлы и 100% полезной инфы. Часть 2: читать и скачать онлайн бесп</t>
+          <t>Сайт не ответил (Timeout).</t>
         </is>
       </c>
       <c r="S47" s="3" t="inlineStr"/>
@@ -4174,18 +4162,14 @@
         </is>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R48" s="3" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S48" s="3" t="inlineStr">
-        <is>
-          <t>B0930d2</t>
-        </is>
-      </c>
+          <t>Сайт не ответил (Timeout).</t>
+        </is>
+      </c>
+      <c r="S48" s="3" t="inlineStr"/>
     </row>
     <row r="49" ht="58" customHeight="1">
       <c r="A49" s="4" t="n">
@@ -4405,7 +4389,7 @@
       </c>
       <c r="R51" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Préparation à l’examen du DELF B2 – Language Learning</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Préparation à l’examen du DELF B2 – Language Learning</t>
         </is>
       </c>
       <c r="S51" s="3" t="inlineStr"/>
@@ -4551,11 +4535,11 @@
         </is>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R53" s="3" t="inlineStr">
         <is>
-          <t>Страницы нет: ответ 200, Ошибка | Не удается получить доступ к сайту.</t>
+          <t>Получена страница ошибки вместо книги. Отсутствие книги не подтверждено, нужна повторная проверка.</t>
         </is>
       </c>
       <c r="S53" s="3" t="inlineStr"/>
@@ -4622,18 +4606,14 @@
       <c r="O54" s="4" t="inlineStr"/>
       <c r="P54" s="4" t="inlineStr"/>
       <c r="Q54" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R54" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S54" s="4" t="inlineStr">
-        <is>
-          <t>Be74d3f</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S54" s="4" t="inlineStr"/>
     </row>
     <row r="55" ht="58" customHeight="1">
       <c r="A55" s="4" t="n">
@@ -4697,14 +4677,18 @@
       <c r="O55" s="4" t="inlineStr"/>
       <c r="P55" s="4" t="inlineStr"/>
       <c r="Q55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R55" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S55" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S55" s="4" t="inlineStr">
+        <is>
+          <t>Bdaf254</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="58" customHeight="1">
       <c r="A56" s="4" t="n">
@@ -4772,7 +4756,7 @@
       </c>
       <c r="R56" s="4" t="inlineStr">
         <is>
-          <t>Название "Бракованный джинн" совпало, но автора из каталога (Ravenna) на странице нет. Нужна проверка человеком.</t>
+          <t>Название "Бракованный джинн" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="S56" s="4" t="inlineStr"/>
@@ -4847,7 +4831,7 @@
       </c>
       <c r="R57" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Занимательные раскраски</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Занимательные раскраски</t>
         </is>
       </c>
       <c r="S57" s="3" t="inlineStr"/>
@@ -5060,18 +5044,14 @@
       <c r="O60" s="4" t="inlineStr"/>
       <c r="P60" s="4" t="inlineStr"/>
       <c r="Q60" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R60" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S60" s="4" t="inlineStr">
-        <is>
-          <t>Be054eb</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S60" s="4" t="inlineStr"/>
     </row>
     <row r="61" ht="58" customHeight="1">
       <c r="A61" s="4" t="n">
@@ -5595,7 +5575,7 @@
       </c>
       <c r="R67" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Переход в 5D. Тайный код для жизни без границ и болезней.: читать и скачать онлайн бесплатно полност</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Переход в 5D. Тайный код для жизни без границ и болезней.: читать и скачать онлайн бесплатно полностью fb2</t>
         </is>
       </c>
       <c r="S67" s="3" t="inlineStr"/>
@@ -5666,14 +5646,18 @@
         </is>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R68" s="3" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S68" s="3" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S68" s="3" t="inlineStr">
+        <is>
+          <t>B4b3214</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="58" customHeight="1">
       <c r="A69" s="4" t="n">
@@ -5737,18 +5721,14 @@
       <c r="O69" s="4" t="inlineStr"/>
       <c r="P69" s="4" t="inlineStr"/>
       <c r="Q69" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R69" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S69" s="4" t="inlineStr">
-        <is>
-          <t>B4b3214</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S69" s="4" t="inlineStr"/>
     </row>
     <row r="70" ht="58" customHeight="1">
       <c r="A70" s="4" t="n">
@@ -5818,14 +5798,18 @@
       </c>
       <c r="P70" s="4" t="inlineStr"/>
       <c r="Q70" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R70" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S70" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S70" s="4" t="inlineStr">
+        <is>
+          <t>Bdaf254</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="58" customHeight="1">
       <c r="A71" s="4" t="n">
@@ -5889,14 +5873,18 @@
       <c r="O71" s="4" t="inlineStr"/>
       <c r="P71" s="4" t="inlineStr"/>
       <c r="Q71" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R71" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S71" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S71" s="4" t="inlineStr">
+        <is>
+          <t>B4b3214</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="58" customHeight="1">
       <c r="A72" s="4" t="n">
@@ -5964,7 +5952,7 @@
       </c>
       <c r="R72" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S72" s="4" t="inlineStr"/>
@@ -6031,18 +6019,14 @@
       <c r="O73" s="4" t="inlineStr"/>
       <c r="P73" s="4" t="inlineStr"/>
       <c r="Q73" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R73" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S73" s="4" t="inlineStr">
-        <is>
-          <t>B144a58</t>
-        </is>
-      </c>
+          <t>Название "(Не)зачёт для птички" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: Daniella. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S73" s="4" t="inlineStr"/>
     </row>
     <row r="74" ht="58" customHeight="1">
       <c r="A74" s="4" t="n">
@@ -6116,7 +6100,7 @@
       </c>
       <c r="R74" s="4" t="inlineStr">
         <is>
-          <t>Название "Бракованный джинн" совпало, но автора из каталога (Ravenna) на странице нет. Нужна проверка человеком.</t>
+          <t>Название "Бракованный джинн" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="S74" s="4" t="inlineStr"/>
@@ -6270,7 +6254,7 @@
       </c>
       <c r="R76" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Книги автора Равенна | LitBox | Равенна - скачать и читать все книги онлайн бесплатно полностью</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Книги автора Равенна | LitBox | Равенна - скачать и читать все книги онлайн бесплатно полностью</t>
         </is>
       </c>
       <c r="S76" s="3" t="inlineStr"/>
@@ -6625,14 +6609,18 @@
       <c r="O81" s="4" t="inlineStr"/>
       <c r="P81" s="4" t="inlineStr"/>
       <c r="Q81" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R81" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S81" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S81" s="4" t="inlineStr">
+        <is>
+          <t>B8b83ea</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="58" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -6785,18 +6773,14 @@
       </c>
       <c r="P83" s="4" t="inlineStr"/>
       <c r="Q83" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R83" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S83" s="4" t="inlineStr">
-        <is>
-          <t>Bf8c90f</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S83" s="4" t="inlineStr"/>
     </row>
     <row r="84" ht="58" customHeight="1">
       <c r="A84" s="4" t="n">
@@ -6866,14 +6850,18 @@
       </c>
       <c r="P84" s="4" t="inlineStr"/>
       <c r="Q84" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R84" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S84" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S84" s="4" t="inlineStr">
+        <is>
+          <t>B8b83ea</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="58" customHeight="1">
       <c r="A85" s="4" t="n">
@@ -7091,7 +7079,7 @@
       </c>
       <c r="R87" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Цена прощения: читать и скачать онлайн бесплатно полностью без сокращений</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Цена прощения: читать и скачать онлайн бесплатно полностью без сокращений</t>
         </is>
       </c>
       <c r="S87" s="3" t="inlineStr"/>
@@ -7166,7 +7154,7 @@
       </c>
       <c r="R88" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Цена прощения: читать и скачать полностью бесплатно онлайн без сокращений FB2</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Цена прощения: читать и скачать полностью бесплатно онлайн без сокращений FB2</t>
         </is>
       </c>
       <c r="S88" s="3" t="inlineStr"/>
@@ -7241,7 +7229,7 @@
       </c>
       <c r="R89" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Цена прощения: читать и скачать онлайн бесплатно полностью fb2</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Цена прощения: читать и скачать онлайн бесплатно полностью fb2</t>
         </is>
       </c>
       <c r="S89" s="3" t="inlineStr"/>
@@ -7316,7 +7304,7 @@
       </c>
       <c r="R90" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Цена прощения: читать и скачать полностью онлайн бесплатно без сокращений FB2</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Цена прощения: читать и скачать полностью онлайн бесплатно без сокращений FB2</t>
         </is>
       </c>
       <c r="S90" s="3" t="inlineStr"/>
@@ -7610,14 +7598,18 @@
       <c r="O94" s="4" t="inlineStr"/>
       <c r="P94" s="4" t="inlineStr"/>
       <c r="Q94" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R94" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S94" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S94" s="4" t="inlineStr">
+        <is>
+          <t>B14dce4</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="58" customHeight="1">
       <c r="A95" s="4" t="n">
@@ -7687,14 +7679,18 @@
       </c>
       <c r="P95" s="4" t="inlineStr"/>
       <c r="Q95" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R95" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S95" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S95" s="4" t="inlineStr">
+        <is>
+          <t>B14dce4</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="58" customHeight="1">
       <c r="A96" s="4" t="n">
@@ -7762,18 +7758,14 @@
       </c>
       <c r="P96" s="4" t="inlineStr"/>
       <c r="Q96" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R96" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S96" s="4" t="inlineStr">
-        <is>
-          <t>Ba025f1</t>
-        </is>
-      </c>
+          <t>Название "Хозяйка Солнечного поместья" совпало, но автора из каталога (Адриана Дари) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S96" s="4" t="inlineStr"/>
     </row>
     <row r="97" ht="58" customHeight="1">
       <c r="A97" s="4" t="n">
@@ -7837,18 +7829,14 @@
       <c r="O97" s="4" t="inlineStr"/>
       <c r="P97" s="4" t="inlineStr"/>
       <c r="Q97" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R97" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S97" s="4" t="inlineStr">
-        <is>
-          <t>B2899ff</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S97" s="4" t="inlineStr"/>
     </row>
     <row r="98" ht="58" customHeight="1">
       <c r="A98" s="4" t="n">
@@ -7918,18 +7906,14 @@
       </c>
       <c r="P98" s="4" t="inlineStr"/>
       <c r="Q98" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R98" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S98" s="4" t="inlineStr">
-        <is>
-          <t>B2899ff</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S98" s="4" t="inlineStr"/>
     </row>
     <row r="99" ht="58" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -8303,18 +8287,14 @@
       <c r="O103" s="4" t="inlineStr"/>
       <c r="P103" s="4" t="inlineStr"/>
       <c r="Q103" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R103" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S103" s="4" t="inlineStr">
-        <is>
-          <t>B7dd037</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S103" s="4" t="inlineStr"/>
     </row>
     <row r="104" ht="58" customHeight="1">
       <c r="A104" s="4" t="n">
@@ -8692,7 +8672,7 @@
       </c>
       <c r="R108" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S108" s="4" t="inlineStr"/>
@@ -8842,14 +8822,18 @@
       <c r="O110" s="4" t="inlineStr"/>
       <c r="P110" s="4" t="inlineStr"/>
       <c r="Q110" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R110" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S110" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S110" s="4" t="inlineStr">
+        <is>
+          <t>Bbec4dd</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="58" customHeight="1">
       <c r="A111" s="4" t="n">
@@ -8913,18 +8897,14 @@
       <c r="O111" s="4" t="inlineStr"/>
       <c r="P111" s="4" t="inlineStr"/>
       <c r="Q111" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R111" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S111" s="4" t="inlineStr">
-        <is>
-          <t>Bbec4dd</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S111" s="4" t="inlineStr"/>
     </row>
     <row r="112" ht="58" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -8996,7 +8976,7 @@
       </c>
       <c r="R112" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Download Python Testing with pytest by Brian Okken | Python Testing with pytest EPUB</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Download Python Testing with pytest by Brian Okken | Python Testing with pytest EPUB</t>
         </is>
       </c>
       <c r="S112" s="3" t="inlineStr"/>
@@ -9213,14 +9193,18 @@
       <c r="O115" s="4" t="inlineStr"/>
       <c r="P115" s="4" t="inlineStr"/>
       <c r="Q115" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R115" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S115" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S115" s="4" t="inlineStr">
+        <is>
+          <t>Be7cb4c</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="58" customHeight="1">
       <c r="A116" s="4" t="n">
@@ -9438,18 +9422,14 @@
       </c>
       <c r="P118" s="4" t="inlineStr"/>
       <c r="Q118" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R118" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S118" s="4" t="inlineStr">
-        <is>
-          <t>B6f939c</t>
-        </is>
-      </c>
+          <t>Название "Пухленькая Рыженькая" совпало, но автора из каталога (Алекс Мара) на странице нет. На странице указан автор: liv. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S118" s="4" t="inlineStr"/>
     </row>
     <row r="119" ht="58" customHeight="1">
       <c r="A119" s="3" t="n">
@@ -9600,7 +9580,7 @@
       </c>
       <c r="R120" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S120" s="4" t="inlineStr"/>
@@ -9667,18 +9647,14 @@
       <c r="O121" s="4" t="inlineStr"/>
       <c r="P121" s="4" t="inlineStr"/>
       <c r="Q121" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R121" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S121" s="4" t="inlineStr">
-        <is>
-          <t>B8b2feb</t>
-        </is>
-      </c>
+          <t>Название "Девственность по контракту" совпало, но автора из каталога (Алекс Найт) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S121" s="4" t="inlineStr"/>
     </row>
     <row r="122" ht="58" customHeight="1">
       <c r="A122" s="4" t="n">
@@ -9817,7 +9793,7 @@
       </c>
       <c r="R123" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S123" s="4" t="inlineStr"/>
@@ -9884,18 +9860,14 @@
       <c r="O124" s="4" t="inlineStr"/>
       <c r="P124" s="4" t="inlineStr"/>
       <c r="Q124" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R124" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S124" s="4" t="inlineStr">
-        <is>
-          <t>Bc730f2</t>
-        </is>
-      </c>
+          <t>Название "Жена для Синей Бороды" совпало, но автора из каталога (Алекс Найт) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S124" s="4" t="inlineStr"/>
     </row>
     <row r="125" ht="58" customHeight="1">
       <c r="A125" s="4" t="n">
@@ -9959,11 +9931,11 @@
       <c r="O125" s="4" t="inlineStr"/>
       <c r="P125" s="4" t="inlineStr"/>
       <c r="Q125" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R125" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Курс Промтология. Большое руководство по нейросетям [Алекс Промтов] со скидкой 50%</t>
         </is>
       </c>
       <c r="S125" s="4" t="inlineStr"/>
@@ -10190,18 +10162,14 @@
       </c>
       <c r="P128" s="4" t="inlineStr"/>
       <c r="Q128" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R128" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S128" s="4" t="inlineStr">
-        <is>
-          <t>B7dd037</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S128" s="4" t="inlineStr"/>
     </row>
     <row r="129" ht="58" customHeight="1">
       <c r="A129" s="4" t="n">
@@ -10427,18 +10395,14 @@
       </c>
       <c r="P131" s="4" t="inlineStr"/>
       <c r="Q131" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R131" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S131" s="4" t="inlineStr">
-        <is>
-          <t>Bce9a30</t>
-        </is>
-      </c>
+          <t>Название "Тайновидец. Том 9: Повелитель стихий" совпало, но автора из каталога (Алекс Рудин) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S131" s="4" t="inlineStr"/>
     </row>
     <row r="132" ht="58" customHeight="1">
       <c r="A132" s="4" t="n">
@@ -10585,18 +10549,14 @@
       </c>
       <c r="P133" s="4" t="inlineStr"/>
       <c r="Q133" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R133" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S133" s="4" t="inlineStr">
-        <is>
-          <t>Bce9a30</t>
-        </is>
-      </c>
+          <t>Название "Тайновидец. Том 9: Повелитель стихий" совпало, но автора из каталога (Алекс Рудин) на странице нет. На странице указан автор: liv. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S133" s="4" t="inlineStr"/>
     </row>
     <row r="134" ht="58" customHeight="1">
       <c r="A134" s="4" t="n">
@@ -10897,18 +10857,14 @@
       <c r="O137" s="4" t="inlineStr"/>
       <c r="P137" s="4" t="inlineStr"/>
       <c r="Q137" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R137" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S137" s="4" t="inlineStr">
-        <is>
-          <t>Bbd74a3</t>
-        </is>
-      </c>
+          <t>Название "Двойное удовольствие" совпало, но автора из каталога (Алекс Хот) на странице нет. На странице указан автор: Mery. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S137" s="4" t="inlineStr"/>
     </row>
     <row r="138" ht="58" customHeight="1">
       <c r="A138" s="3" t="n">
@@ -11122,18 +11078,14 @@
       <c r="O140" s="4" t="inlineStr"/>
       <c r="P140" s="4" t="inlineStr"/>
       <c r="Q140" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R140" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
-        </is>
-      </c>
-      <c r="S140" s="4" t="inlineStr">
-        <is>
-          <t>Be7cb4c</t>
-        </is>
-      </c>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
+        </is>
+      </c>
+      <c r="S140" s="4" t="inlineStr"/>
     </row>
     <row r="141" ht="58" customHeight="1">
       <c r="A141" s="4" t="n">
@@ -11203,14 +11155,18 @@
       </c>
       <c r="P141" s="4" t="inlineStr"/>
       <c r="Q141" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R141" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S141" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S141" s="4" t="inlineStr">
+        <is>
+          <t>Be7cb4c</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="58" customHeight="1">
       <c r="A142" s="3" t="n">
@@ -11359,18 +11315,14 @@
       </c>
       <c r="P143" s="4" t="inlineStr"/>
       <c r="Q143" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R143" s="4" t="inlineStr">
         <is>
-          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: скачивание epub, fb2, txt; чтение онлайн; кнопка скачивания.</t>
-        </is>
-      </c>
-      <c r="S143" s="4" t="inlineStr">
-        <is>
-          <t>B116af7</t>
-        </is>
-      </c>
+          <t>Название "Будь моим бывшим" совпало, но автора из каталога (Мара Алекс) на странице нет. На странице указан автор: Daniella. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="S143" s="4" t="inlineStr"/>
     </row>
     <row r="144" ht="58" customHeight="1">
       <c r="A144" s="4" t="n">
@@ -11440,11 +11392,11 @@
       </c>
       <c r="P144" s="4" t="inlineStr"/>
       <c r="Q144" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R144" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Курс Промтология. Большое руководство по нейросетям [Алекс Промтов] со скидкой 50%</t>
         </is>
       </c>
       <c r="S144" s="4" t="inlineStr"/>
@@ -11602,7 +11554,7 @@
       </c>
       <c r="R146" s="3" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Егерь: назад в СССР: читать и скачать онлайн бесплатно полностью без сокращений</t>
+          <t>Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Егерь: назад в СССР: читать и скачать онлайн бесплатно полностью без сокращений</t>
         </is>
       </c>
       <c r="S146" s="3" t="inlineStr"/>
@@ -11823,14 +11775,18 @@
       <c r="O149" s="4" t="inlineStr"/>
       <c r="P149" s="4" t="inlineStr"/>
       <c r="Q149" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R149" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
-        </is>
-      </c>
-      <c r="S149" s="4" t="inlineStr"/>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: кнопка скачивания; ссылка скрыта до регистрации.</t>
+        </is>
+      </c>
+      <c r="S149" s="4" t="inlineStr">
+        <is>
+          <t>B3ff35a</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="58" customHeight="1">
       <c r="A150" s="4" t="n">
@@ -11973,7 +11929,7 @@
       </c>
       <c r="R151" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Получен экран загрузки вместо содержимого. Нужна проверка в браузере.</t>
         </is>
       </c>
       <c r="S151" s="4" t="inlineStr"/>
@@ -15779,7 +15735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15892,555 +15848,539 @@
     </row>
     <row r="4" ht="58" customHeight="1">
       <c r="A4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Findroid</t>
+          <t>DIGITAL ZEN</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Гнев Империи. Книга 1</t>
+          <t>ПРОМПТ SUNO.COM энциклопедия и полное руководство по составлению промпта.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>https://musportal.pro/track/1756600919-findroid-glava-01-gnev-imperii-kniga-1</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>тип ebook, а ссылка похожа на аудио</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr"/>
+          <t>https://skladchik.tv/threads/prompt-suno-com-ehnciklopedija-i-polnoe-rukovodstvo-po-sostavleniju-prompta-ddigital-zen.489299/</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "ПРОМПТ SUNO.COM энциклопедия и полное руководство по составлению промпта." совпало, но автора из каталога (DIGITAL ZEN) на странице нет. Нужна проверка человеком.</t>
+        </is>
+      </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>на какие форматы есть права: текст, аудио</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Ася Исай</t>
+          <t>Findroid</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Измена. Хочу твоего мужа</t>
+          <t>Гнев Империи. Книга 1</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>https://kniganet.ru/romani/izmena-hochu-tvoego-muzha/</t>
+          <t>https://musportal.pro/track/1756600919-findroid-glava-01-gnev-imperii-kniga-1</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>это же название есть у других авторов: Галина Колоскова, Мария Авенская</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Измена. Хочу твоего мужа" совпало, но автора из каталога (Ася Исай, Галина Колоскова, Мария Авенская) на странице нет. Нужна проверка человеком.</t>
-        </is>
-      </c>
+          <t>тип ebook, а ссылка похожа на аудио</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>ID книги или ISBN, чтобы различать одноимённые книги; варианты имени автора и псевдонимы</t>
+          <t>на какие форматы есть права: текст, аудио</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="4" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Disciplimit</t>
+          <t>Ася Исай</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Дисциплина ставок. Инструменты системного игрока. Журнал, банкролл, психология, рутина</t>
+          <t>Измена. Хочу твоего мужа</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>https://dolinakursov.ru/threads/disciplimit-disciplimit-sistema-kontrolja-reshenij.59305/</t>
+          <t>https://kniganet.ru/romani/izmena-hochu-tvoego-muzha/</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr"/>
+          <t>это же название есть у других авторов: Галина Колоскова, Мария Авенская</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): ИИ-проверка: Название совпадает, но указанный на странице автор Оксана Алексаева отсутствует среди кандидатов.</t>
+        </is>
+      </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="4" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ira Kiba</t>
+          <t>DIGITAL ZEN</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Кармические узлы в натальной карте</t>
+          <t>ПРОМПТ SUNO.COM энциклопедия и полное руководство по составлению промпта.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>https://astro-babylon.ru/biblioteca-main/karmicheskaya-astrologiya.html</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
-        </is>
-      </c>
+          <t>https://s4.skladchik.tv/threads/prompt-suno-com-ehnciklopedija-i-polnoe-rukovodstvo-po-sostavleniju-prompta-ddigital-zen.489299/</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Кармическая астрология | Книги по кармической астрологии</t>
+          <t>страница не подтвердила книгу (статус 2): Название "ПРОМПТ SUNO.COM энциклопедия и полное руководство по составлению промпта." совпало, но автора из каталога (DIGITAL ZEN) на странице нет. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="4" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Jana Denole Яна Деноль</t>
+          <t>Disciplimit</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Gaunerinnen</t>
+          <t>Дисциплина ставок. Инструменты системного игрока. Журнал, банкролл, психология, рутина</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>https://read.xbook.life/books_gaunerinnen_67131402</t>
+          <t>https://dolinakursov.ru/threads/disciplimit-disciplimit-sistema-kontrolja-reshenij.59305/</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>в поле автора два написания, латиницей и кириллицей</t>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr"/>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>основное имя автора и варианты написания</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
         </is>
       </c>
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Armine Grigoryan</t>
+          <t>Helga Duran</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ставка на любовь</t>
+          <t>Тарский горячий твой</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>https://mp3deer.cc/mp3/armine-grigoryan-erevani-sirun-txa</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 0% слов); тип ebook, а ссылка похожа на аудио</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr"/>
+          <t>https://listaibuk.com/sovremennie-lyubovnie-romani/tarskiy-goryachiy-tvoy/</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Тарский горячий твой" совпало, но автора из каталога (Helga Duran) на странице нет. На странице указан автор: Daniella. Нужна проверка человеком.</t>
+        </is>
+      </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; на какие форматы есть права: текст, аудио</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="4" t="n">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Lanpirot</t>
+          <t>Ira Kiba</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Позывной «Хоттабыч»#6. Аватар "Х"</t>
+          <t>Кармические узлы в натальной карте</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>https://free-kniga.ru/priklyucheniya/pozyvnoy-hottabych-7-avatar-h-ch-2/</t>
+          <t>https://astro-babylon.ru/biblioteca-main/karmicheskaya-astrologiya.html</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>номер тома или части в адресе другой: в названии 6</t>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>на странице другая книга: Lanpirot. Позывной «Хоттабыч»#7. Аватар "Х" (ч.2)</t>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Кармическая астрология | Книги по кармической астрологии</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>серия и номер тома отдельными полями; подтверждение правообладателя, к какой книге относится ссылка</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="4" t="n">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Lanpirot</t>
+          <t>Jana Denole Яна Деноль</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Позывной «Хоттабыч»#9. Исчадие Кромки (ч. 2)</t>
+          <t>Gaunerinnen</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>https://readtoday.ru/priklyucheniya/pozyvnoy-hottabych-9-ischadie-kromki-ch-2/</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 0): Страницы нет: ответ 404, Страница не найдена - ReadToday | 404.</t>
-        </is>
-      </c>
+          <t>https://read.xbook.life/books_gaunerinnen_67131402</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>в поле автора два написания, латиницей и кириллицей</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>не нужны: страница удалена, ссылку можно закрыть</t>
+          <t>основное имя автора и варианты написания</t>
         </is>
       </c>
     </row>
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="4" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Larisa Lubimova</t>
+          <t>Armine Grigoryan</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>ОГЭ-2026 по английскому. Лайфхаки, фейлы и 100% полезной инфы Секреты письменного ОГЭ: от ошибок к совершенству Практические советы по улучшению навыков письма и грамматики.</t>
+          <t>Ставка на любовь</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>https://librain.ru/nauka-i-obrazovanie/oge-2026-po-angliiskomu-laifxaki-feily-i-100-poleznoi-infy-cast-2</t>
+          <t>https://mp3deer.cc/mp3/armine-grigoryan-erevani-sirun-txa</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 39% слов)</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: ОГЭ-2026 по английскому. Лайфхаки, фейлы и 100% полезной инфы. Часть 2: читать и скачать онлайн бесп</t>
-        </is>
-      </c>
+          <t>адрес страницы не похож на название (совпало 0% слов); тип ebook, а ссылка похожа на аудио</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; на какие форматы есть права: текст, аудио</t>
         </is>
       </c>
     </row>
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="4" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Елена Полярная</t>
+          <t>Lanpirot</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Измена. Я вас верну</t>
+          <t>Позывной «Хоттабыч»#6. Аватар "Х"</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>https://librain.ru/index.php/detektivy/izmena-ia-vas-vernu</t>
+          <t>https://free-kniga.ru/priklyucheniya/pozyvnoy-hottabych-7-avatar-h-ch-2/</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>это же название есть у других авторов: Арина Салай, Оксана Алексаева, Полина Рей</t>
+          <t>номер тома или части в адресе другой: в названии 6</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>на странице другая книга: Оксана Алексаева. Измена. Я вас верну</t>
+          <t>на странице другая книга: Lanpirot. Позывной «Хоттабыч»#7. Аватар "Х" (ч.2)</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>ID книги или ISBN, чтобы различать одноимённые книги; подтверждение правообладателя, к какой книге относится ссылка</t>
+          <t>серия и номер тома отдельными полями; подтверждение правообладателя, к какой книге относится ссылка</t>
         </is>
       </c>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="4" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Lilit Khachinyan</t>
+          <t>Lanpirot</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Guide de préparation à la production orale du DELF B2</t>
+          <t>Позывной «Хоттабыч»#9. Исчадие Кромки (ч. 2)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>https://languagelearning.site/french/preparation-a-lexamen-du-delf-b2-2/</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 40% слов)</t>
-        </is>
-      </c>
+          <t>https://readtoday.ru/priklyucheniya/pozyvnoy-hottabych-9-ischadie-kromki-ch-2/</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Préparation à l’examen du DELF B2 – Language Learning</t>
+          <t>страница не подтвердила книгу (статус 0): Страницы нет: ответ 404, Страница не найдена - ReadToday | 404.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>не нужны: страница удалена, ссылку можно закрыть</t>
         </is>
       </c>
     </row>
     <row r="15" ht="58" customHeight="1">
       <c r="A15" s="4" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Lost In Space</t>
+          <t>Larisa Lubimova</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Наследник, которого не должно быть</t>
+          <t>ОГЭ-2026 по английскому. Лайфхаки, фейлы и 100% полезной инфы Секреты письменного ОГЭ: от ошибок к совершенству Практические советы по улучшению навыков письма и грамматики.</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>https://mp3deer.cc/mp3/%D1%81%D1%83%D0%BF%D0%B5%D1%80-%D0%B0%D1%83%D0%B4%D0%B8%D0%BE%D0%BA%D0%BD%D0%B8%D0%B3%D0%B0-%D0%BD%D0%B0%D1%81%D0%BB%D0%B5%D0%B4%D0%BD%D0%B8%D0%BA-%D0%BA%D0%BE%D1%82%D0%BE%D1%80%D0%BE%D0%B3%D0%BE-%D0%BD%D0%B5-%D0%B4%D0%BE%D0%BB%D0%B6%D0%BD%D0%BE-%D0%B1%D1%8B%D1%82%D1%8C</t>
+          <t>https://librain.ru/nauka-i-obrazovanie/oge-2026-po-angliiskomu-laifxaki-feily-i-100-poleznoi-infy-cast-2</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>тип ebook, а ссылка похожа на аудио</t>
+          <t>адрес страницы не похож на название (совпало 39% слов)</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>на какие форматы есть права: текст, аудио</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
         </is>
       </c>
     </row>
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Lucy Zen</t>
+          <t>Елена Полярная</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Автономия</t>
+          <t>Измена. Я вас верну</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>https://skladmk.online/product/energiya-zhizni-lucy-zen/</t>
+          <t>https://librain.ru/index.php/detektivy/izmena-ia-vas-vernu</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 0): Страницы нет: ответ 200, Ошибка | Не удается получить доступ к сайту.</t>
-        </is>
-      </c>
+          <t>это же название есть у других авторов: Арина Салай, Оксана Алексаева, Полина Рей</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; не нужны: страница удалена, ссылку можно закрыть</t>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
         </is>
       </c>
     </row>
     <row r="17" ht="58" customHeight="1">
       <c r="A17" s="4" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Lilit Khachinyan</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Бракованный джинн</t>
+          <t>Guide de préparation à la production orale du DELF B2</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>https://kniganet.ru/fentezi/brakovannyy-dzhinn/</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr"/>
+          <t>https://languagelearning.site/french/preparation-a-lexamen-du-delf-b2-2/</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>адрес страницы не похож на название (совпало 40% слов)</t>
+        </is>
+      </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Бракованный джинн" совпало, но автора из каталога (Ravenna) на странице нет. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Préparation à l’examen du DELF B2 – Language Learning</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>варианты имени автора и псевдонимы</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="18" ht="58" customHeight="1">
       <c r="A18" s="4" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>MILA NENKA</t>
+          <t>Lost In Space</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Маленькие заботы. Мини-раскраска для самых маленьких</t>
+          <t>Наследник, которого не должно быть</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>https://2ivdel.tvoysadik.ru/?section_id=98</t>
+          <t>https://mp3deer.cc/mp3/%D1%81%D1%83%D0%BF%D0%B5%D1%80-%D0%B0%D1%83%D0%B4%D0%B8%D0%BE%D0%BA%D0%BD%D0%B8%D0%B3%D0%B0-%D0%BD%D0%B0%D1%81%D0%BB%D0%B5%D0%B4%D0%BD%D0%B8%D0%BA-%D0%BA%D0%BE%D1%82%D0%BE%D1%80%D0%BE%D0%B3%D0%BE-%D0%BD%D0%B5-%D0%B4%D0%BE%D0%BB%D0%B6%D0%BD%D0%BE-%D0%B1%D1%8B%D1%82%D1%8C</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Занимательные раскраски</t>
-        </is>
-      </c>
+          <t>тип ebook, а ссылка похожа на аудио</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника; проверить, та ли ссылка указана для книги</t>
+          <t>на какие форматы есть права: текст, аудио</t>
         </is>
       </c>
     </row>
     <row r="19" ht="58" customHeight="1">
       <c r="A19" s="4" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Mind Wave</t>
+          <t>Lucy Zen</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Левитация. Путь к внутренней свободе</t>
+          <t>Автономия</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>https://mx-style.net/product/levitacziya-put-k-vnutrennej-svobode-mind-wave/</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 0): Страницы нет: ответ 404, Ошибка | Не удается получить доступ к сайту.</t>
-        </is>
-      </c>
+          <t>https://skladmk.online/product/energiya-zhizni-lucy-zen/</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>не нужны: страница удалена, ссылку можно закрыть</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
         </is>
       </c>
     </row>
     <row r="20" ht="58" customHeight="1">
       <c r="A20" s="4" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Nika Nika</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Кето-рецепты</t>
+          <t>Бракованный джинн</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>https://librain.ru/zdorove/keto-recepty</t>
+          <t>https://kniganet.ru/fentezi/brakovannyy-dzhinn/</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr"/>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Кето-рецепты" совпало, но автора из каталога (Nika Nika) на странице нет. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Бракованный джинн" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -16451,263 +16391,267 @@
     </row>
     <row r="21" ht="58" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Nina BROD</t>
+          <t>MILA NENKA</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Тишина</t>
+          <t>Маленькие заботы. Мини-раскраска для самых маленьких</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>https://aknigi24.com/book/tisina-spokoistvie-v-mire-polnom-suma-tit-nat-xan-nikosho</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr"/>
+          <t>https://2ivdel.tvoysadik.ru/?section_id=98</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
+        </is>
+      </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Тишина" совпало, но автора из каталога (Nina BROD) на странице нет. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Занимательные раскраски</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>варианты имени автора и псевдонимы</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="22" ht="58" customHeight="1">
       <c r="A22" s="4" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Findroid</t>
+          <t>Mind Wave</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Гнев Империи. Книга 1</t>
+          <t>Левитация. Путь к внутренней свободе</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>https://musportal.pro/track/1756600919-findroid-glava-01-gnev-imperii-kniga-1</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>тип ebook, а ссылка похожа на аудио</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr"/>
+          <t>https://mx-style.net/product/levitacziya-put-k-vnutrennej-svobode-mind-wave/</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страницы нет: ответ 404, Ошибка | Не удается получить доступ к сайту.</t>
+        </is>
+      </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>на какие форматы есть права: текст, аудио</t>
+          <t>не нужны: страница удалена, ссылку можно закрыть</t>
         </is>
       </c>
     </row>
     <row r="23" ht="58" customHeight="1">
       <c r="A23" s="4" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Ominayashi</t>
+          <t>Nika Nika</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Пять звезд. Часть 5</t>
+          <t>Кето-рецепты</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>https://knigi.ebooker.online/book/42876144-kniga-pyat-zvezd.-chast-5</t>
+          <t>https://librain.ru/zdorove/keto-recepty</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr"/>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книга найдена в заголовке, автор совпал. Книга упомянута, но скачать, читать или слушать нельзя.</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Кето-рецепты" совпало, но автора из каталога (Nika Nika) на странице нет. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>не нужны: размещения нет</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="24" ht="58" customHeight="1">
       <c r="A24" s="4" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Quartz Y</t>
+          <t>Nina BROD</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Переход в 5D измерение. Просветление. Методичка</t>
+          <t>Тишина</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>https://librain.ru/putesestviia-i-geografiia/perexod-v-5d-tainyi-kod-dlia-zizni-bez-granic-i-boleznei</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 25% слов)</t>
-        </is>
-      </c>
+          <t>https://aknigi24.com/book/tisina-spokoistvie-v-mire-polnom-suma-tit-nat-xan-nikosho</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Переход в 5D. Тайный код для жизни без границ и болезней.: читать и скачать онлайн бесплатно полност</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Тишина" совпало, но автора из каталога (Nina BROD) на странице нет. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="25" ht="58" customHeight="1">
       <c r="A25" s="4" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Rais Ais Gu</t>
+          <t>Findroid</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Искусство простоты Навести порядок в вещах, делах и мыслях</t>
+          <t>Гнев Империи. Книга 1</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>https://skladchik.tv/threads/nastroit-svoj-mozg-ne-mozhesh-sosredotochitsja-zabyvaesh-vsjo-na-svete-tjanesh-s-resheniem-rais-gu.450854/</t>
+          <t>https://musportal.pro/track/1756600919-findroid-glava-01-gnev-imperii-kniga-1</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+          <t>тип ebook, а ссылка похожа на аудио</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+          <t>на какие форматы есть права: текст, аудио</t>
         </is>
       </c>
     </row>
     <row r="26" ht="58" customHeight="1">
       <c r="A26" s="4" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Ominayashi</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Бракованный джинн</t>
+          <t>Пять звезд. Часть 5</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>https://kniganet.ru/fentezi/brakovannyy-dzhinn/</t>
+          <t>https://knigi.ebooker.online/book/42876144-kniga-pyat-zvezd.-chast-5</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr"/>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Бракованный джинн" совпало, но автора из каталога (Ravenna) на странице нет. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 0): Книга найдена в заголовке, автор совпал. Книга упомянута, но скачать, читать или слушать нельзя.</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>варианты имени автора и псевдонимы</t>
+          <t>не нужны: размещения нет</t>
         </is>
       </c>
     </row>
     <row r="27" ht="58" customHeight="1">
       <c r="A27" s="4" t="n">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Vector</t>
+          <t>Quartz Y</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Констебль. Том III</t>
+          <t>Переход в 5D измерение. Просветление. Методичка</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>https://ruslibrary.org/fantastika-fjentezi/418-vector-sbornik-knig.html</t>
+          <t>https://librain.ru/putesestviia-i-geografiia/perexod-v-5d-tainyi-kod-dlia-zizni-bez-granic-i-boleznei</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr"/>
+          <t>адрес страницы не похож на название (совпало 25% слов)</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Переход в 5D. Тайный код для жизни без границ и болезней.: читать и скачать онлайн бесплатно полностью fb2</t>
+        </is>
+      </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="28" ht="58" customHeight="1">
       <c r="A28" s="4" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Rais Ais Gu</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Медовичок</t>
+          <t>Искусство простоты Навести порядок в вещах, делах и мыслях</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>https://litbox.pro/tag/ravenna/</t>
+          <t>https://skladchik.tv/threads/nastroit-svoj-mozg-ne-mozhesh-sosredotochitsja-zabyvaesh-vsjo-na-svete-tjanesh-s-resheniem-rais-gu.450854/</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Книги автора Равенна | LitBox | Равенна - скачать и читать все книги онлайн бесплатно полностью</t>
+          <t>на странице другая книга: Rais Ais Gu. Настроить свой мозг. Не можешь сосредоточиться? Забываешь всё на свете? Тянешь с решением?</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника; проверить, та ли ссылка указана для книги</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; подтверждение правообладателя, к какой книге относится ссылка</t>
         </is>
       </c>
     </row>
     <row r="29" ht="58" customHeight="1">
       <c r="A29" s="4" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -16716,18 +16660,18 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Медовичок</t>
+          <t>(Не)зачёт для птички</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>https://litseries.ru/romany/medovichok-533516/</t>
+          <t>https://litbox.pro/sovremennie-lyubovnie-romani/ne-zachyot-dlya-ptichki/</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Медовичок" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: Юлия Ши. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 2): Название "(Не)зачёт для птички" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: Daniella. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -16738,73 +16682,69 @@
     </row>
     <row r="30" ht="58" customHeight="1">
       <c r="A30" s="4" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Галина Колоскова</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Измена. Хочу твоего мужа</t>
+          <t>Бракованный джинн</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>https://mir-chitki.com/romany/8472-izmena-hochu-tvoego-muzha.html</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>это же название есть у других авторов: Ася Исай, Мария Авенская</t>
-        </is>
-      </c>
+          <t>https://kniganet.ru/fentezi/brakovannyy-dzhinn/</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Измена. Хочу твоего мужа" совпало, но автора из каталога (Ася Исай, Галина Колоскова, Мария Авенская) на странице нет. На странице указан автор: Оксана Алексаева. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Бракованный джинн" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>ID книги или ISBN, чтобы различать одноимённые книги; варианты имени автора и псевдонимы</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="31" ht="58" customHeight="1">
       <c r="A31" s="4" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Медовичок</t>
+          <t>Констебль. Том III</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>https://pro-books.ru/liubovnye-romany/medovicok</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Медовичок" совпало, но автора из каталога (Ravenna) на странице нет. Нужна проверка человеком.</t>
-        </is>
-      </c>
+          <t>https://ruslibrary.org/fantastika-fjentezi/418-vector-sbornik-knig.html</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>варианты имени автора и псевдонимы</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника</t>
         </is>
       </c>
     </row>
     <row r="32" ht="58" customHeight="1">
       <c r="A32" s="4" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
@@ -16818,195 +16758,187 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>https://readtoday.ru/romany/medovichok-311872/</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr"/>
+          <t>https://litbox.pro/tag/ravenna/</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
+        </is>
+      </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Медовичок" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: Юлия Ши. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Книги автора Равенна | LitBox | Равенна - скачать и читать все книги онлайн бесплатно полностью</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>варианты имени автора и псевдонимы</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="33" ht="58" customHeight="1">
       <c r="A33" s="4" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Vector</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Констебль. Том III</t>
+          <t>Медовичок</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>https://ruslibrary.org/fantastika-fjentezi/418-vector-sbornik-knig.html</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr"/>
+          <t>https://litseries.ru/romany/medovichok-533516/</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Медовичок" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: Юлия Ши. Нужна проверка человеком.</t>
+        </is>
+      </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="34" ht="58" customHeight="1">
       <c r="A34" s="4" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Авее Лав</t>
+          <t>Галина Колоскова</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Ценадоверия</t>
+          <t>Измена. Хочу твоего мужа</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>https://free-kniga.ru/romany/tsena-proscheniya-147884/</t>
+          <t>https://mir-chitki.com/romany/8472-izmena-hochu-tvoego-muzha.html</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+          <t>это же название есть у других авторов: Ася Исай, Мария Авенская</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Цена прощения: читать и скачать онлайн бесплатно полностью без сокращений</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Измена. Хочу твоего мужа" совпало, но автора из каталога (Ася Исай, Галина Колоскова, Мария Авенская) на странице нет. На странице указан автор: Оксана Алексаева. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги; варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="35" ht="58" customHeight="1">
       <c r="A35" s="4" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Авее Лав</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Ценадоверия</t>
+          <t>Медовичок</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>https://gigabooks.ru/romany/tsena-proscheniya-686299/</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
-        </is>
-      </c>
+          <t>https://pro-books.ru/liubovnye-romany/medovicok</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Цена прощения: читать и скачать полностью бесплатно онлайн без сокращений FB2</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Медовичок" совпало, но автора из каталога (Ravenna) на странице нет. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="36" ht="58" customHeight="1">
       <c r="A36" s="4" t="n">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Авее Лав</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Ценадоверия</t>
+          <t>Медовичок</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>https://librain.ru/sovremennye-liubovnye-romany/cena-proshheniia</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
-        </is>
-      </c>
+          <t>https://readtoday.ru/romany/medovichok-311872/</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr"/>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Цена прощения: читать и скачать онлайн бесплатно полностью fb2</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Медовичок" совпало, но автора из каталога (Ravenna) на странице нет. На странице указан автор: Юлия Ши. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="37" ht="58" customHeight="1">
       <c r="A37" s="4" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Авее Лав</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Ценадоверия</t>
+          <t>Констебль. Том III</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>https://litseries.ru/romany/tsena-proscheniya-203253/</t>
+          <t>https://ruslibrary.org/fantastika-fjentezi/418-vector-sbornik-knig.html</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Цена прощения: читать и скачать полностью онлайн бесплатно без сокращений FB2</t>
-        </is>
-      </c>
+          <t>адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника</t>
         </is>
       </c>
     </row>
     <row r="38" ht="58" customHeight="1">
       <c r="A38" s="4" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
@@ -17020,24 +16952,28 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>https://free-kniga.ru/boevik/cena-doveriia/</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr"/>
+          <t>https://free-kniga.ru/romany/tsena-proscheniya-147884/</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Ценадоверия" совпало, но автора из каталога (Авее Лав) на странице нет. На странице указан автор: ИИ Текст. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Цена прощения: читать и скачать онлайн бесплатно полностью без сокращений</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>варианты имени автора и псевдонимы</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="39" ht="58" customHeight="1">
       <c r="A39" s="4" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
@@ -17051,7 +16987,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>https://wav-library.net/sovremennaia-proza/cena-proshheniia</t>
+          <t>https://gigabooks.ru/romany/tsena-proscheniya-686299/</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -17059,57 +16995,69 @@
           <t>адрес страницы не похож на название (совпало 0% слов)</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Цена прощения: читать и скачать полностью бесплатно онлайн без сокращений FB2</t>
+        </is>
+      </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="40" ht="58" customHeight="1">
       <c r="A40" s="4" t="n">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Алекс Ключевской</t>
+          <t>Авее Лав</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Тёмный маг. Книга 1. Неведомый путь</t>
+          <t>Ценадоверия</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>https://knigoline.ru/tyomnyy-mag-kniga-1-nevedomyy-put-4375/</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr"/>
+          <t>https://librain.ru/sovremennye-liubovnye-romany/cena-proshheniia</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Книга найдена в заголовке, автор совпал. Есть ссылки на магазин и признаки чтения или скачивания; назначение ссылок нужно проверить.</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr"/>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Цена прощения: читать и скачать онлайн бесплатно полностью fb2</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="58" customHeight="1">
       <c r="A41" s="4" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Алекс Мара</t>
+          <t>Авее Лав</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Разведенаипрекрасна</t>
+          <t>Ценадоверия</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>https://free-kniga.ru/yumor/razvedena-i-prekrasna-379393/</t>
+          <t>https://litseries.ru/romany/tsena-proscheniya-203253/</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -17117,140 +17065,140 @@
           <t>адрес страницы не похож на название (совпало 0% слов)</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Цена прощения: читать и скачать полностью онлайн бесплатно без сокращений FB2</t>
+        </is>
+      </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="42" ht="58" customHeight="1">
       <c r="A42" s="4" t="n">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Алекс Коган</t>
+          <t>Авее Лав</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Изучаем pytest: От основ до продвинутых техник тестирования в Python</t>
+          <t>Ценадоверия</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>https://bibliophile.top/index.php?threads/11672/</t>
+          <t>https://free-kniga.ru/boevik/cena-doveriia/</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книга найдена в заголовке, автор совпал. Книга упомянута, но скачать, читать или слушать нельзя.</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Ценадоверия" совпало, но автора из каталога (Авее Лав) на странице нет. На странице указан автор: ИИ Текст. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>не нужны: размещения нет</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="43" ht="58" customHeight="1">
       <c r="A43" s="4" t="n">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Алекс Ключевской</t>
+          <t>Адриана Дари</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>13-й демон Асмодея. Том 2</t>
+          <t>Хозяйка Солнечного поместья</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>https://knigoline.ru/13-y-demon-asmodeya-tom-2-9093/</t>
+          <t>https://kniganet.ru/drama/nenuzhnaya-istinnaya-drakona-hozyayka-solnechnogo-pomestya/</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Книга найдена в заголовке, автор совпал. Есть ссылки на магазин и признаки чтения или скачивания; назначение ссылок нужно проверить.</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr"/>
+          <t>страница не подтвердила книгу (статус 2): Название "Хозяйка Солнечного поместья" совпало, но автора из каталога (Адриана Дари) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>варианты имени автора и псевдонимы</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="58" customHeight="1">
       <c r="A44" s="4" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Алекс Коган</t>
+          <t>Авее Лав</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Изучаем pytest: От основ до продвинутых техник тестирования в Python</t>
+          <t>Ценадоверия</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>https://zlib.pub/book/python-testing-with-pytest-3g998v3in3tg</t>
+          <t>https://wav-library.net/sovremennaia-proza/cena-proshheniia</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 29% слов)</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Download Python Testing with pytest by Brian Okken | Python Testing with pytest EPUB</t>
-        </is>
-      </c>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
         </is>
       </c>
     </row>
     <row r="45" ht="58" customHeight="1">
       <c r="A45" s="4" t="n">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Алекс Крамер</t>
+          <t>Алекс Ключевской</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Уличная еда: рецепты блюд современного стрит-фуда</t>
+          <t>Тёмный маг. Книга 1. Неведомый путь</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>https://zoboko.com/book/rm9vg3d3/</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
-        </is>
-      </c>
+          <t>https://knigoline.ru/tyomnyy-mag-kniga-1-nevedomyy-put-4375/</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Книга найдена в заголовке, автор совпал. Есть ссылки на магазин и признаки чтения или скачивания; назначение ссылок нужно проверить.</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr"/>
     </row>
     <row r="46" ht="58" customHeight="1">
       <c r="A46" s="4" t="n">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
@@ -17264,7 +17212,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>https://readtoday.ru/yumor/razvedena-i-prekrasna-727057/</t>
+          <t>https://free-kniga.ru/yumor/razvedena-i-prekrasna-379393/</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -17281,270 +17229,704 @@
     </row>
     <row r="47" ht="58" customHeight="1">
       <c r="A47" s="4" t="n">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Оксана Алексаева</t>
+          <t>Алекс Коган</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Измена. Я вас верну</t>
+          <t>Изучаем pytest: От основ до продвинутых техник тестирования в Python</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>https://booksfb2.com/liubovnye-romany/izmena-ia-vas-vernu</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>это же название есть у других авторов: Арина Салай, Елена Полярная, Полина Рей</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr"/>
+          <t>https://bibliophile.top/index.php?threads/11672/</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Книга найдена в заголовке, автор совпал. Книга упомянута, но скачать, читать или слушать нельзя.</t>
+        </is>
+      </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+          <t>не нужны: размещения нет</t>
         </is>
       </c>
     </row>
     <row r="48" ht="58" customHeight="1">
       <c r="A48" s="4" t="n">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Мария Авенская</t>
+          <t>Алекс Ключевской</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Измена. Хочу твоего мужа</t>
+          <t>13-й демон Асмодея. Том 2</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>https://knigi.fun/31487-izmena-hochu-tvoego-mugha.html</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>это же название есть у других авторов: Ася Исай, Галина Колоскова</t>
-        </is>
-      </c>
+          <t>https://knigoline.ru/13-y-demon-asmodeya-tom-2-9093/</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Измена. Хочу твоего мужа" совпало, но автора из каталога (Ася Исай, Галина Колоскова, Мария Авенская) на странице нет. На странице указан автор: Оксана Алексаева. Нужна проверка человеком.</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>ID книги или ISBN, чтобы различать одноимённые книги; варианты имени автора и псевдонимы</t>
-        </is>
-      </c>
+          <t>страница не подтвердила книгу (статус 2): Книга найдена в заголовке, автор совпал. Есть ссылки на магазин и признаки чтения или скачивания; назначение ссылок нужно проверить.</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr"/>
     </row>
     <row r="49" ht="58" customHeight="1">
       <c r="A49" s="4" t="n">
-        <v>138</v>
+        <v>112</v>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Арина Салай</t>
+          <t>Алекс Коган</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Измена. Я вас верну</t>
+          <t>Изучаем pytest: От основ до продвинутых техник тестирования в Python</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>https://wav-library.net/proza/izmena-ia-vas-vernu</t>
+          <t>https://zlib.pub/book/python-testing-with-pytest-3g998v3in3tg</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>это же название есть у других авторов: Елена Полярная, Оксана Алексаева, Полина Рей</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr"/>
+          <t>адрес страницы не похож на название (совпало 29% слов)</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Download Python Testing with pytest by Brian Okken | Python Testing with pytest EPUB</t>
+        </is>
+      </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; проверить, та ли ссылка указана для книги</t>
         </is>
       </c>
     </row>
     <row r="50" ht="58" customHeight="1">
       <c r="A50" s="4" t="n">
-        <v>139</v>
+        <v>117</v>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Дари Адриана</t>
+          <t>Алекс Крамер</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Хозяйка таверны "У Черных скал"</t>
+          <t>Уличная еда: рецепты блюд современного стрит-фуда</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>https://readtoday.ru/priklyucheniya/oklevetannaya-zhena-drakona-hozyayka-taverny-u-chernyh-skal-945787/</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>страница не подтвердила книгу (статус 0): Страницы нет: ответ 404, Страница не найдена - ReadToday | 404.</t>
-        </is>
-      </c>
+          <t>https://zoboko.com/book/rm9vg3d3/</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr"/>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>не нужны: страница удалена, ссылку можно закрыть</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
         </is>
       </c>
     </row>
     <row r="51" ht="58" customHeight="1">
       <c r="A51" s="4" t="n">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Мария Авенская</t>
+          <t>Алекс Мара</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Измена. Хочу твоего мужа</t>
+          <t>Пухленькая Рыженькая</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>https://knigi.fun/31487-izmena-hochu-tvoego-mugha.html</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>это же название есть у других авторов: Ася Исай, Галина Колоскова</t>
-        </is>
-      </c>
+          <t>https://libvi.ru/yumor/puhlenkaya-ryzhenkaya/</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr"/>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 2): Название "Измена. Хочу твоего мужа" совпало, но автора из каталога (Ася Исай, Галина Колоскова, Мария Авенская) на странице нет. На странице указан автор: Оксана Алексаева. Нужна проверка человеком.</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Пухленькая Рыженькая" совпало, но автора из каталога (Алекс Мара) на странице нет. На странице указан автор: liv. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>ID книги или ISBN, чтобы различать одноимённые книги; варианты имени автора и псевдонимы</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="52" ht="58" customHeight="1">
       <c r="A52" s="4" t="n">
-        <v>145</v>
+        <v>119</v>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Полина Рей</t>
+          <t>Алекс Мара</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Измена. Я вас верну</t>
+          <t>Разведенаипрекрасна</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>https://pro-books.ru/proza/izmena-ia-vas-vernu</t>
+          <t>https://readtoday.ru/yumor/razvedena-i-prekrasna-727057/</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>это же название есть у других авторов: Арина Салай, Елена Полярная, Оксана Алексаева</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>на странице другая книга: Оксана Алексаева. Измена. Я вас верну</t>
-        </is>
-      </c>
+          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr"/>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>ID книги или ISBN, чтобы различать одноимённые книги; подтверждение правообладателя, к какой книге относится ссылка</t>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
         </is>
       </c>
     </row>
     <row r="53" ht="58" customHeight="1">
       <c r="A53" s="4" t="n">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Рудин Алекс</t>
+          <t>Алекс Найт</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Егерь-2: Назад в СССР</t>
+          <t>Девственность по контракту</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>https://free-kniga.ru/priklyucheniya/eger-nazad-v-sssr-669853/</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>номер тома или части в адресе другой: в названии 2</t>
-        </is>
-      </c>
+          <t>https://kniganet.ru/fentezi/devstvennost-po-kontraktu/</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>страница не подтвердила книгу (статус 0): Книг из каталога на странице нет. Страница про: Егерь: назад в СССР: читать и скачать онлайн бесплатно полностью без сокращений</t>
+          <t>страница не подтвердила книгу (статус 2): Название "Девственность по контракту" совпало, но автора из каталога (Алекс Найт) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>серия и номер тома отдельными полями; проверить, та ли ссылка указана для книги</t>
+          <t>варианты имени автора и псевдонимы</t>
         </is>
       </c>
     </row>
     <row r="54" ht="58" customHeight="1">
       <c r="A54" s="4" t="n">
-        <v>147</v>
+        <v>124</v>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Егорова Надежда</t>
+          <t>Алекс Найт</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Ночь на Лысой горе. Где забытые боги слышат</t>
+          <t>Жена для Синей Бороды</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>https://lllit.ru/ezoterika/noc-na-lysoi-gore-gde-zabytye-bogi-slysat</t>
+          <t>https://kniganet.ru/romani/zhena-dlya-siney-borody/</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr"/>
       <c r="F54" s="4" t="inlineStr">
         <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Жена для Синей Бороды" совпало, но автора из каталога (Алекс Найт) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>варианты имени автора и псевдонимы</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="58" customHeight="1">
+      <c r="A55" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Алекс Промтов</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Промтология. Большое руководство по нейросетям: от основ ИИ до готовых решений</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>https://s3.skladchinabiz.app/threads/promtologija-bolshoe-rukovodstvo-po-nejrosetjam-aleks-promtov.465616/</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Курс Промтология. Большое руководство по нейросетям [Алекс Промтов] со скидкой 50%</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>проверить, та ли ссылка указана для книги</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="58" customHeight="1">
+      <c r="A56" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Оксана Алексаева</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Я вас верну</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>https://booksfb2.com/liubovnye-romany/izmena-ia-vas-vernu</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>это же название есть у других авторов: Арина Салай, Елена Полярная, Полина Рей</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr"/>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="58" customHeight="1">
+      <c r="A57" s="4" t="n">
+        <v>127</v>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Мария Авенская</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Хочу твоего мужа</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>https://knigi.fun/31487-izmena-hochu-tvoego-mugha.html</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>это же название есть у других авторов: Ася Исай, Галина Колоскова</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Измена. Хочу твоего мужа" совпало, но автора из каталога (Ася Исай, Галина Колоскова, Мария Авенская) на странице нет. На странице указан автор: Оксана Алексаева. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги; варианты имени автора и псевдонимы</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="58" customHeight="1">
+      <c r="A58" s="4" t="n">
+        <v>131</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Алекс Рудин</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Тайновидец. Том 9: Повелитель стихий</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>https://kniganet.ru/priklyucheniya/taynovidets-tom-9-povelitel-stihiy/</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Тайновидец. Том 9: Повелитель стихий" совпало, но автора из каталога (Алекс Рудин) на странице нет. На странице указан автор: autoposter. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>варианты имени автора и псевдонимы</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="58" customHeight="1">
+      <c r="A59" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Алекс Рудин</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Тайновидец. Том 9: Повелитель стихий</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>https://libvi.ru/fentezi/taynovidets-tom-9-povelitel-stihiy/</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Тайновидец. Том 9: Повелитель стихий" совпало, но автора из каталога (Алекс Рудин) на странице нет. На странице указан автор: liv. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>варианты имени автора и псевдонимы</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="58" customHeight="1">
+      <c r="A60" s="4" t="n">
+        <v>137</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Алекс Хот</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Двойное удовольствие</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>https://knigo-lub.ru/erotika/dvoynoe-udovolstvie/</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Двойное удовольствие" совпало, но автора из каталога (Алекс Хот) на странице нет. На странице указан автор: Mery. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>варианты имени автора и псевдонимы</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="58" customHeight="1">
+      <c r="A61" s="4" t="n">
+        <v>138</v>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Арина Салай</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Я вас верну</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>https://wav-library.net/proza/izmena-ia-vas-vernu</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>это же название есть у других авторов: Елена Полярная, Оксана Алексаева, Полина Рей</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="58" customHeight="1">
+      <c r="A62" s="4" t="n">
+        <v>139</v>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Дари Адриана</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Хозяйка таверны "У Черных скал"</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>https://readtoday.ru/priklyucheniya/oklevetannaya-zhena-drakona-hozyayka-taverny-u-chernyh-skal-945787/</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страницы нет: ответ 404, Страница не найдена - ReadToday | 404.</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>не нужны: страница удалена, ссылку можно закрыть</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="58" customHeight="1">
+      <c r="A63" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Мария Авенская</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Хочу твоего мужа</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>https://knigi.fun/31487-izmena-hochu-tvoego-mugha.html</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>это же название есть у других авторов: Ася Исай, Галина Колоскова</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Измена. Хочу твоего мужа" совпало, но автора из каталога (Ася Исай, Галина Колоскова, Мария Авенская) на странице нет. На странице указан автор: Оксана Алексаева. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги; варианты имени автора и псевдонимы</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="58" customHeight="1">
+      <c r="A64" s="4" t="n">
+        <v>143</v>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Мара Алекс</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Будь моим бывшим</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>https://litbox.pro/sovremennie-lyubovnie-romani/bud-moim-bivshim/</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 2): Название "Будь моим бывшим" совпало, но автора из каталога (Мара Алекс) на странице нет. На странице указан автор: Daniella. Нужна проверка человеком.</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>варианты имени автора и псевдонимы</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="58" customHeight="1">
+      <c r="A65" s="4" t="n">
+        <v>144</v>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Алекс Промтов</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Промтология. Большое руководство по нейросетям: от основ ИИ до готовых решений</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>https://skladchinabiz.app/threads/promtologija-bolshoe-rukovodstvo-po-nejrosetjam-aleks-promtov.465616/</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Курс Промтология. Большое руководство по нейросетям [Алекс Промтов] со скидкой 50%</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>проверить, та ли ссылка указана для книги</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="58" customHeight="1">
+      <c r="A66" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Полина Рей</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Я вас верну</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>https://pro-books.ru/proza/izmena-ia-vas-vernu</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>это же название есть у других авторов: Арина Салай, Елена Полярная, Оксана Алексаева</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>на странице другая книга: Оксана Алексаева. Измена. Я вас верну</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги; подтверждение правообладателя, к какой книге относится ссылка</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="58" customHeight="1">
+      <c r="A67" s="4" t="n">
+        <v>146</v>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Рудин Алекс</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Егерь-2: Назад в СССР</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>https://free-kniga.ru/priklyucheniya/eger-nazad-v-sssr-669853/</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>номер тома или части в адресе другой: в названии 2</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>страница не подтвердила книгу (статус 0): Страница прочитана, но совпадение с каталогом не найдено. Обнаружено: Егерь: назад в СССР: читать и скачать онлайн бесплатно полностью без сокращений</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>серия и номер тома отдельными полями; проверить, та ли ссылка указана для книги</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="58" customHeight="1">
+      <c r="A68" s="4" t="n">
+        <v>147</v>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Егорова Надежда</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Ночь на Лысой горе. Где забытые боги слышат</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>https://lllit.ru/ezoterika/noc-na-lysoi-gore-gde-zabytye-bogi-slysat</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
           <t>страница не подтвердила книгу (статус 0): Страницы нет: редирект на главную.</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t>не нужны: страница удалена, ссылку можно закрыть</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G54"/>
+  <autoFilter ref="A1:G68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17752,7 +18134,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>заголовок: Разреши любить. Позволь мне быть рядом. Книга 2 Анна Джейн; тип: application/pdf</t>
+          <t>заголовок: Разреши любить. Позволь мне быть рядом. Книга 2 Анна Джейн; автор на странице: Анна Джейн; тип: application/pdf</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
@@ -17762,7 +18144,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>Книг из каталога на странице нет. Страница про: Разреши любить. Позволь мне быть рядом. Книга 2 Анна Джейн</t>
+          <t>PDF найден и прочитан, но совпадение с каталогом не найдено. Обнаружено: Разреши любить. Позволь мне быть рядом. Книга 2 Анна Джейн</t>
         </is>
       </c>
     </row>
@@ -17815,7 +18197,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>заголовок: Системный разведчик. Инфильтрация. Дилогия, Юрич Валерий - читать онлайн без регистрации</t>
+          <t>заголовок: Системный разведчик. Инфильтрация. Дилогия, Юрич Валерий - читать онлайн без регистрации; автор на странице: Юрич Валерий</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -18053,7 +18435,7 @@
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
@@ -18067,17 +18449,17 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>заголовок: Ярость Вечных: скачать fb2, epub, pdf, txt | Антон Карелин; автор на странице: Антон Карелин; ИИ: решение уточнено, цитаты проверены</t>
+          <t>заголовок: Ярость Вечных: скачать fb2, epub, pdf, txt | Антон Карелин; автор на странице: Антон Карелин; ИИ: ИИ не дал проверяемого ответа, сохранено решение правил</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>Антон Карелин. Ярость Вечных</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>ИИ-проверка: Есть совпадение названия и автора, но размещение книги не подтверждено: на сайте предлагается лишь покупка платной версии на партнёрском ресурсе.</t>
+          <t>Книга найдена в заголовке, автор совпал. Есть ссылки на магазин и признаки чтения или скачивания; назначение ссылок нужно проверить.</t>
         </is>
       </c>
     </row>
@@ -18193,7 +18575,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>заголовок: Ясновидеть может каждый или как развить в себе сверхспособности, Хайр Хелен, книга полностью, читать бесплатно без сокращений</t>
+          <t>заголовок: Ясновидеть может каждый или как развить в себе сверхспособности, Хайр Хелен, книга полностью, читать бесплатно без сокращений; автор на странице: Хайр Хелен</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -18242,27 +18624,31 @@
         </is>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I11" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>текст книги прямо на странице</t>
+        </is>
+      </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>200, нет содержимого</t>
+          <t>200, ok</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>заголовок: Загрузка — Библибоба</t>
+          <t>заголовок: Читать Я-Мир. Инструкция по переходу от внутренней гадости к истинной радости (Игорь Леонидович Науменко) бесплатно и полностью – книга жанра "Наука, ; автор на странице: Игорь Леонидович Науменко; загрузка: браузер Playwright</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>Игорь Леонидович Науменко. Я-Мир. Инструкция по переходу от внутренней гадости к истинной радости</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>Сайт не отдал содержимое без браузера: проверка на бота или страница собирается скриптом.</t>
+          <t>Книга найдена в заголовке, автор совпал. Признаки размещения: текст книги прямо на странице.</t>
         </is>
       </c>
     </row>
@@ -18278,7 +18664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18321,22 +18707,22 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+          <t>dolinakursov.ru/threads/disciplimit</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Проверить, что ссылка ведёт на эту книгу, а не на другой товар</t>
+          <t>URL содержит «sistema-kontrolja-reshenij», не совпадает с названием книги. Уточните привязку.</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Полный URL и подтверждение названия со страницы</t>
+          <t>подтверждение, что это тот же материал</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>ИИ: deepseek-v4.1-flash; цитата проверена</t>
+          <t>ИИ: qwen-3.8-flash; цитата проверена</t>
         </is>
       </c>
     </row>
@@ -18346,22 +18732,22 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>тип ebook, а ссылка похожа на аудио</t>
+          <t>mp3deer.cc/mp3/armine-grigoryan</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Уточнить формат издания и соответствует ли ссылка ему</t>
+          <t>Ссылка ведёт на аудиоплеер, а тип записи - ebook. Также в slug армянское название.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Полный URL, формат и обложка или описание страницы</t>
+          <t>ссылка на текст или смена типа на audio</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>ИИ: deepseek-v4.1-flash; цитата проверена</t>
+          <t>ИИ: qwen-3.8-flash; цитата проверена</t>
         </is>
       </c>
     </row>
@@ -18371,22 +18757,22 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>тип ebook, а ссылка похожа на аудио</t>
+          <t>musportal.pro/track/1756600919</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Сверить формат с типом записи перед публикацией</t>
+          <t>URL страницы трека, а тип - ebook. Вероятно, ссылка на аудиокнигу.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Полный URL и явное указание формата</t>
+          <t>ссылка на текст или смена типа на audio</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>ИИ: deepseek-v4.1-flash; цитата проверена</t>
+          <t>ИИ: qwen-3.8-flash; цитата проверена</t>
         </is>
       </c>
     </row>
@@ -18396,127 +18782,852 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>это же название есть у других авторов: Галина Колоскова, Мария Авенская</t>
+          <t>Измена. Хочу твоего мужа</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Проверить автора и издание, не сливать книги разных авторов</t>
+          <t>Название дублируется у других авторов. Проверьте, не одно ли это произведение под разными именами.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>ISBN или издательские данные для каждой версии</t>
+          <t>данные об авторстве или ISBN</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>ИИ: deepseek-v4.1-flash; цитата проверена</t>
+          <t>ИИ: qwen-3.8-flash; цитата проверена</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="4" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>адрес страницы не похож на название (совпало 0% слов)</t>
+          <t>dolinakursov.ru/threads/disciplimit</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Проверить соответствие ссылки названию и автору</t>
+          <t>Дублирует строку 2. Подтвердите, что это отдельная запись или уберите повтор.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Полный URL и название со страницы</t>
+          <t>решение о дубликате</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>ИИ: deepseek-v4.1-flash; цитата проверена</t>
+          <t>ИИ: qwen-3.8-flash; цитата проверена</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="4" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>в поле автора два написания, латиницей и кириллицей</t>
+          <t>astro-babylon.ru/biblioteca-main/</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Уточнить, это один автор или псевдоним, не склеивать записи</t>
+          <t>Slug «karmicheskaya-astrologiya» шире заголовка. Уточните, конкретна ли страница.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Ссылка на профиль автора и подтверждение написания</t>
+          <t>конкретная страница книги</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>ИИ: deepseek-v4.1-flash; цитата проверена</t>
+          <t>ИИ: qwen-3.8-flash; цитата проверена</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="4" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>номер тома или части в адресе другой: в названии 6</t>
+          <t>Jana Denole Яна Деноль</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Проверить номер тома в названии и на странице издания</t>
+          <t>В поле автора два написания. Выберите одно каноническое, другое перенесите в псевдонимы.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Полный URL и номер тома с обложки</t>
+          <t>каноническое написание имени</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>ИИ: deepseek-v4.1-flash; цитата проверена</t>
+          <t>ИИ: qwen-3.8-flash; цитата проверена</t>
         </is>
       </c>
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>mp3deer.cc/mp3/armine-grigoryan</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Дублирует строку 7 с той же проблемой: ebook-тип при аудио-URL. Подтвердите или уберите.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>решение о дубликате и типе</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: qwen-3.8-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Позывной «Хоттабыч»#6. Аватар "Х"</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Проверить соответствие номера части в названии и в адресе страницы</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Точное название части и номер тома от правообладателя</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: glm-5.3-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>адрес страницы не похож на название (совпало 39% слов)</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Сверить ссылку и слишком длинное название, возможно это сборник</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Полный URL и структура названия из источника</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>ИИ: deepseek-v4.1-flash; цитата проверена</t>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Лайфхаки, фейлы и 100% полезной инфы</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Название не совпадает с адресом, возможно склеены две книги; уточнить одну книгу или серию</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Оригинальное название и ссылка со страницы книги</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: glm-5.3-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Я вас верну</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Одно название у нескольких авторов; сверить автора и обложку с первоисточником</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждение авторства и ISBN или ID издания</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: glm-5.3-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Guide de préparation à la production orale</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Адрес содержит пометку -2, возможен дубликат страницы; проверить каноническую ссылку</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Канонический URL и оригинальное название издания</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: glm-5.3-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Наследник, которого не должно быть</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Тип ebook, а ссылка ведёт на аудио-раздел; уточнить формат издания</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждение формата и корректная ссылка на текст</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: glm-5.3-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Автономия</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Адрес ведёт на другой товар того же автора; сверить название с карточкой товара</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Название по странице магазина и ID товара</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: glm-5.3-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Мини-раскраска для самых маленьких</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Ссылка похожа на страницу раздела, а не книги; запросить прямую ссылку на издание</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Прямой URL карточки книги</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: glm-5.3-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Гнев Империи. Книга 1</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Тип ebook, но ссылка на аудиотрек; проверить формат и источник</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Подтверждение формата и ссылка на ebook-издание</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>ИИ: glm-5.3-flash; цитата проверена</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Переход в 5D измерение. Просветление. Методичка</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 25% слов)</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Искусство простоты Навести порядок в вещах, делах и мыслях</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Констебль. Том III</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Медовичок</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Хочу твоего мужа</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: это же название есть у других авторов: Ася Исай, Мария Авенская</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Констебль. Том III</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов); похоже на страницу тега, раздела или сборника, а не одной книги</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки; ссылка на страницу конкретной книги или состав сборника</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Ценадоверия</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>88</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Ценадоверия</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Ценадоверия</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Правила: ответ ИИ не подтверждён или API недоступен</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Ценадоверия</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Правила: ответ ИИ не подтверждён или API недоступен</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="58" customHeight="1">
+      <c r="A28" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Ценадоверия</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Правила: ответ ИИ не подтверждён или API недоступен</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="A29" s="4" t="n">
+        <v>102</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Разведенаипрекрасна</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Правила: ответ ИИ не подтверждён или API недоступен</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="58" customHeight="1">
+      <c r="A30" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Изучаем pytest: От основ до продвинутых техник тестирования в Python</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 29% слов)</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Правила: ответ ИИ не подтверждён или API недоступен</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="58" customHeight="1">
+      <c r="A31" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Уличная еда: рецепты блюд современного стрит-фуда</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Правила: ответ ИИ не подтверждён или API недоступен</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="58" customHeight="1">
+      <c r="A32" s="4" t="n">
+        <v>119</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Разведенаипрекрасна</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: адрес страницы не похож на название (совпало 0% слов)</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>ID книги у правообладателя (артикул или ISBN) для каждой ссылки</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Правила: ответ ИИ не подтверждён или API недоступен</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="58" customHeight="1">
+      <c r="A33" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Я вас верну</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: это же название есть у других авторов: Арина Салай, Елена Полярная, Полина Рей</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Правила: ответ ИИ не подтверждён или API недоступен</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="58" customHeight="1">
+      <c r="A34" s="4" t="n">
+        <v>127</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Хочу твоего мужа</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: это же название есть у других авторов: Ася Исай, Галина Колоскова</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="58" customHeight="1">
+      <c r="A35" s="4" t="n">
+        <v>138</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Я вас верну</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: это же название есть у других авторов: Елена Полярная, Оксана Алексаева, Полина Рей</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="58" customHeight="1">
+      <c r="A36" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Хочу твоего мужа</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: это же название есть у других авторов: Ася Исай, Галина Колоскова</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="58" customHeight="1">
+      <c r="A37" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Измена. Я вас верну</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: это же название есть у других авторов: Арина Салай, Елена Полярная, Оксана Алексаева</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>ID книги или ISBN, чтобы различать одноимённые книги</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="58" customHeight="1">
+      <c r="A38" s="4" t="n">
+        <v>146</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Егерь-2: Назад в СССР</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Проверить: номер тома или части в адресе другой: в названии 2</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>серия и номер тома отдельными полями</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Правила: превышено время ожидания ИИ</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:E38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>